<commit_message>
chore: auto-scrape data 2026-10-12
</commit_message>
<xml_diff>
--- a/data/FI_data.xlsx
+++ b/data/FI_data.xlsx
@@ -1264,12 +1264,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating outside of US will be settled next-day under IAT processing in US</t>
+          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating within US and for amount above 1 Mn USD will be credited to beneficiary on next-business day Payments originating outside of US will be settled next-day under IAT processing in US</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -19279,12 +19279,12 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating outside of US will be settled next-day under IAT processing in US</t>
+          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating within US and for amount above 1 Mn USD will be credited to beneficiary on next-business day Payments originating outside of US will be settled next-day under IAT processing in US</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="Q171" t="inlineStr">
@@ -19294,7 +19294,7 @@
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="S171" t="inlineStr">
@@ -19304,7 +19304,7 @@
       </c>
       <c r="T171" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="U171" t="inlineStr">
@@ -19314,7 +19314,7 @@
       </c>
       <c r="V171" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="W171" t="inlineStr">
@@ -35202,12 +35202,12 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating outside of US will be settled next-day under IAT processing in US</t>
+          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating within US and for amount above 1 Mn USD will be credited to beneficiary on next-business day Payments originating outside of US will be settled next-day under IAT processing in US</t>
         </is>
       </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="Q314" t="inlineStr">
@@ -35217,7 +35217,7 @@
       </c>
       <c r="R314" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="S314" t="inlineStr">
@@ -35227,7 +35227,7 @@
       </c>
       <c r="T314" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="U314" t="inlineStr">
@@ -35237,7 +35237,7 @@
       </c>
       <c r="V314" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="W314" t="inlineStr">
@@ -38710,12 +38710,12 @@
       </c>
       <c r="O346" t="inlineStr">
         <is>
-          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating outside of US will be settled next-day under IAT processing in US</t>
+          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating within US and for amount above 1 Mn USD will be credited to beneficiary on next-business day Payments originating outside of US will be settled next-day under IAT processing in US</t>
         </is>
       </c>
       <c r="P346" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="Q346" t="inlineStr">
@@ -38725,7 +38725,7 @@
       </c>
       <c r="R346" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="S346" t="inlineStr">
@@ -38735,7 +38735,7 @@
       </c>
       <c r="T346" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="U346" t="inlineStr">
@@ -38745,7 +38745,7 @@
       </c>
       <c r="V346" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="W346" t="inlineStr">
@@ -50281,12 +50281,12 @@
       </c>
       <c r="O449" t="inlineStr">
         <is>
-          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating outside of US will be settled next-day under IAT processing in US</t>
+          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating within US and for amount above 1 Mn USD will be credited to beneficiary on next-business day Payments originating outside of US will be settled next-day under IAT processing in US</t>
         </is>
       </c>
       <c r="P449" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="Q449" t="inlineStr">
@@ -50296,7 +50296,7 @@
       </c>
       <c r="R449" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="S449" t="inlineStr">
@@ -50306,7 +50306,7 @@
       </c>
       <c r="T449" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="U449" t="inlineStr">
@@ -50316,7 +50316,7 @@
       </c>
       <c r="V449" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="W449" t="inlineStr">
@@ -51819,12 +51819,12 @@
       </c>
       <c r="O463" t="inlineStr">
         <is>
-          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating outside of US will be settled next-day under IAT processing in US</t>
+          <t>USD ACH payouts can also be done to below countries if the ACH code is supported as per regulator guidelines. - U. S. Virgin Islands , Guam American Samoa , The Northern Mariana Islands. Payments originating within US and for amount above 1 Mn USD will be credited to beneficiary on next-business day Payments originating outside of US will be settled next-day under IAT processing in US</t>
         </is>
       </c>
       <c r="P463" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="Q463" t="inlineStr">
@@ -51834,7 +51834,7 @@
       </c>
       <c r="R463" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="S463" t="inlineStr">
@@ -51844,7 +51844,7 @@
       </c>
       <c r="T463" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="U463" t="inlineStr">
@@ -51854,7 +51854,7 @@
       </c>
       <c r="V463" t="inlineStr">
         <is>
-          <t>USD 1,000,000</t>
+          <t>USD 9,999,999</t>
         </is>
       </c>
       <c r="W463" t="inlineStr">

</xml_diff>